<commit_message>
data: fill 149 missing examples from supplied workbook
</commit_message>
<xml_diff>
--- a/shared/words/E1_单词汇总.xlsx
+++ b/shared/words/E1_单词汇总.xlsx
@@ -521,6 +521,11 @@
           <t>words/einheit1/lernen.mp3</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sophie und ich lernen Deutsch.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -624,6 +629,11 @@
           <t>words/einheit1/gehen.mp3</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Er geht langsam.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -646,6 +656,11 @@
           <t>words/einheit1/danken.mp3</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ich danke dir für die Hilfe.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1324,6 +1339,11 @@
           <t>words/einheit1/Käse.mp3</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Der Käse ist aus Deutschland.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1393,6 +1413,11 @@
           <t>words/einheit1/Hut.mp3</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Der Hut ist schön.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1573,6 +1598,11 @@
           <t>words/einheit1/Schüler.mp3</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Was macht der Schüler?</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1605,6 +1635,11 @@
           <t>words/einheit1/Schülerin.mp3</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Die Schülerin lernt Deutsch.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1933,6 +1968,11 @@
           <t>words/einheit1/Spiegel.mp3</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Der Spiegel ist modern.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2076,6 +2116,11 @@
           <t>words/einheit1/Lehrerin.mp3</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sie ist Lehrerin.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2337,6 +2382,11 @@
           <t>words/einheit1/wie.mp3</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wie heißen Sie?</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2359,6 +2409,11 @@
           <t>words/einheit1/auch.mp3</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ich komme auch aus China.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2597,6 +2652,11 @@
           <t>words/einheit1/dann.mp3</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dann verabschieden sie sich.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2617,6 +2677,11 @@
       <c r="F66" t="inlineStr">
         <is>
           <t>words/einheit1/gleich.mp3</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ich komme gleich.</t>
         </is>
       </c>
     </row>

</xml_diff>